<commit_message>
E_diffuse  was measured for calibration
</commit_message>
<xml_diff>
--- a/DMX_Dimming_Curve.xlsx
+++ b/DMX_Dimming_Curve.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Aksu\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Documents\berk\roombrightening\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B14EEBC-D072-49D9-9551-231B7FE75309}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19DDEB53-1C9C-481D-9585-D5930CBC8462}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1845" yWindow="-15870" windowWidth="25440" windowHeight="15270" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Diffuse" sheetId="1" r:id="rId1"/>
@@ -150,7 +150,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -178,6 +178,12 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -530,7 +536,9 @@
       <c r="D3" s="3">
         <v>0</v>
       </c>
-      <c r="E3" s="3"/>
+      <c r="E3" s="10">
+        <v>0</v>
+      </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="4">
@@ -545,7 +553,9 @@
       <c r="D4" s="5">
         <v>143</v>
       </c>
-      <c r="E4" s="5"/>
+      <c r="E4" s="11">
+        <v>4.9000000000000004</v>
+      </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="2">
@@ -560,7 +570,9 @@
       <c r="D5" s="3">
         <v>31</v>
       </c>
-      <c r="E5" s="3"/>
+      <c r="E5" s="10">
+        <v>9.94</v>
+      </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="4">
@@ -575,7 +587,9 @@
       <c r="D6" s="5">
         <v>174</v>
       </c>
-      <c r="E6" s="5"/>
+      <c r="E6" s="11">
+        <v>14.89</v>
+      </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="2">
@@ -590,7 +604,9 @@
       <c r="D7" s="3">
         <v>61</v>
       </c>
-      <c r="E7" s="3"/>
+      <c r="E7" s="10">
+        <v>19.600000000000001</v>
+      </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="4">
@@ -605,7 +621,9 @@
       <c r="D8" s="5">
         <v>205</v>
       </c>
-      <c r="E8" s="5"/>
+      <c r="E8" s="11">
+        <v>24.5</v>
+      </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="2">
@@ -620,7 +638,9 @@
       <c r="D9" s="3">
         <v>92</v>
       </c>
-      <c r="E9" s="3"/>
+      <c r="E9" s="10">
+        <v>29.44</v>
+      </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="4">
@@ -635,7 +655,9 @@
       <c r="D10" s="5">
         <v>235</v>
       </c>
-      <c r="E10" s="5"/>
+      <c r="E10" s="11">
+        <v>34.33</v>
+      </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" s="2">
@@ -650,7 +672,9 @@
       <c r="D11" s="3">
         <v>123</v>
       </c>
-      <c r="E11" s="3"/>
+      <c r="E11" s="10">
+        <v>39.200000000000003</v>
+      </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" s="4">
@@ -665,7 +689,9 @@
       <c r="D12" s="5">
         <v>10</v>
       </c>
-      <c r="E12" s="5"/>
+      <c r="E12" s="11">
+        <v>44</v>
+      </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" s="2">
@@ -680,7 +706,9 @@
       <c r="D13" s="3">
         <v>154</v>
       </c>
-      <c r="E13" s="3"/>
+      <c r="E13" s="10">
+        <v>48.8</v>
+      </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" s="4">
@@ -695,7 +723,9 @@
       <c r="D14" s="5">
         <v>41</v>
       </c>
-      <c r="E14" s="5"/>
+      <c r="E14" s="11">
+        <v>53.6</v>
+      </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" s="2">
@@ -710,7 +740,9 @@
       <c r="D15" s="3">
         <v>184</v>
       </c>
-      <c r="E15" s="3"/>
+      <c r="E15" s="10">
+        <v>58.4</v>
+      </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" s="4">
@@ -725,7 +757,9 @@
       <c r="D16" s="5">
         <v>72</v>
       </c>
-      <c r="E16" s="5"/>
+      <c r="E16" s="11">
+        <v>63.22</v>
+      </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="2">
@@ -740,7 +774,9 @@
       <c r="D17" s="3">
         <v>215</v>
       </c>
-      <c r="E17" s="3"/>
+      <c r="E17" s="10">
+        <v>67.900000000000006</v>
+      </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="4">
@@ -755,7 +791,9 @@
       <c r="D18" s="5">
         <v>102</v>
       </c>
-      <c r="E18" s="5"/>
+      <c r="E18" s="11">
+        <v>72.599999999999994</v>
+      </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="2">
@@ -770,7 +808,9 @@
       <c r="D19" s="3">
         <v>246</v>
       </c>
-      <c r="E19" s="3"/>
+      <c r="E19" s="10">
+        <v>77.3</v>
+      </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" s="4">
@@ -785,7 +825,9 @@
       <c r="D20" s="5">
         <v>133</v>
       </c>
-      <c r="E20" s="5"/>
+      <c r="E20" s="11">
+        <v>81.900000000000006</v>
+      </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" s="2">
@@ -800,7 +842,9 @@
       <c r="D21" s="3">
         <v>20</v>
       </c>
-      <c r="E21" s="3"/>
+      <c r="E21" s="10">
+        <v>86.6</v>
+      </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" s="4">
@@ -815,7 +859,9 @@
       <c r="D22" s="5">
         <v>164</v>
       </c>
-      <c r="E22" s="5"/>
+      <c r="E22" s="11">
+        <v>89.5</v>
+      </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" s="2">
@@ -830,7 +876,9 @@
       <c r="D23" s="3">
         <v>51</v>
       </c>
-      <c r="E23" s="3"/>
+      <c r="E23" s="10">
+        <v>94.1</v>
+      </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" s="4">
@@ -845,7 +893,9 @@
       <c r="D24" s="5">
         <v>194</v>
       </c>
-      <c r="E24" s="5"/>
+      <c r="E24" s="11">
+        <v>98.5</v>
+      </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" s="2">
@@ -860,7 +910,9 @@
       <c r="D25" s="3">
         <v>82</v>
       </c>
-      <c r="E25" s="3"/>
+      <c r="E25" s="10">
+        <v>102.9</v>
+      </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" s="4">
@@ -875,7 +927,9 @@
       <c r="D26" s="5">
         <v>225</v>
       </c>
-      <c r="E26" s="5"/>
+      <c r="E26" s="11">
+        <v>107.33</v>
+      </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" s="2">
@@ -890,7 +944,9 @@
       <c r="D27" s="3">
         <v>112</v>
       </c>
-      <c r="E27" s="3"/>
+      <c r="E27" s="10">
+        <v>111.8</v>
+      </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" s="4">
@@ -905,7 +961,9 @@
       <c r="D28" s="5">
         <v>0</v>
       </c>
-      <c r="E28" s="5"/>
+      <c r="E28" s="11">
+        <v>116.2</v>
+      </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" s="2">
@@ -920,7 +978,9 @@
       <c r="D29" s="3">
         <v>143</v>
       </c>
-      <c r="E29" s="3"/>
+      <c r="E29" s="10">
+        <v>120.6</v>
+      </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" s="4">
@@ -935,7 +995,9 @@
       <c r="D30" s="5">
         <v>30</v>
       </c>
-      <c r="E30" s="5"/>
+      <c r="E30" s="11">
+        <v>125</v>
+      </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" s="2">
@@ -950,7 +1012,9 @@
       <c r="D31" s="3">
         <v>174</v>
       </c>
-      <c r="E31" s="3"/>
+      <c r="E31" s="10">
+        <v>129.30000000000001</v>
+      </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" s="4">
@@ -965,7 +1029,9 @@
       <c r="D32" s="5">
         <v>61</v>
       </c>
-      <c r="E32" s="5"/>
+      <c r="E32" s="11">
+        <v>133.6</v>
+      </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" s="2">
@@ -980,7 +1046,9 @@
       <c r="D33" s="3">
         <v>204</v>
       </c>
-      <c r="E33" s="3"/>
+      <c r="E33" s="10">
+        <v>137.80000000000001</v>
+      </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" s="4">
@@ -995,7 +1063,9 @@
       <c r="D34" s="5">
         <v>92</v>
       </c>
-      <c r="E34" s="5"/>
+      <c r="E34" s="11">
+        <v>142</v>
+      </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" s="2">
@@ -1010,7 +1080,9 @@
       <c r="D35" s="3">
         <v>235</v>
       </c>
-      <c r="E35" s="3"/>
+      <c r="E35" s="10">
+        <v>146.30000000000001</v>
+      </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36" s="4">
@@ -1025,7 +1097,9 @@
       <c r="D36" s="5">
         <v>123</v>
       </c>
-      <c r="E36" s="5"/>
+      <c r="E36" s="11">
+        <v>150.5</v>
+      </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37" s="2">
@@ -1040,7 +1114,9 @@
       <c r="D37" s="3">
         <v>10</v>
       </c>
-      <c r="E37" s="3"/>
+      <c r="E37" s="10">
+        <v>154.80000000000001</v>
+      </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38" s="4">
@@ -1055,7 +1131,9 @@
       <c r="D38" s="5">
         <v>153</v>
       </c>
-      <c r="E38" s="5"/>
+      <c r="E38" s="11">
+        <v>159</v>
+      </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A39" s="2">
@@ -1070,7 +1148,9 @@
       <c r="D39" s="3">
         <v>41</v>
       </c>
-      <c r="E39" s="3"/>
+      <c r="E39" s="10">
+        <v>163.1</v>
+      </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40" s="4">
@@ -1085,7 +1165,9 @@
       <c r="D40" s="5">
         <v>184</v>
       </c>
-      <c r="E40" s="5"/>
+      <c r="E40" s="11">
+        <v>167.3</v>
+      </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A41" s="2">
@@ -1100,7 +1182,9 @@
       <c r="D41" s="3">
         <v>71</v>
       </c>
-      <c r="E41" s="3"/>
+      <c r="E41" s="10">
+        <v>171.5</v>
+      </c>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A42" s="4">
@@ -1115,7 +1199,9 @@
       <c r="D42" s="5">
         <v>215</v>
       </c>
-      <c r="E42" s="5"/>
+      <c r="E42" s="11">
+        <v>175.7</v>
+      </c>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A43" s="2">
@@ -1130,7 +1216,9 @@
       <c r="D43" s="3">
         <v>102</v>
       </c>
-      <c r="E43" s="3"/>
+      <c r="E43" s="10">
+        <v>179.8</v>
+      </c>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A44" s="4">
@@ -1145,7 +1233,9 @@
       <c r="D44" s="5">
         <v>245</v>
       </c>
-      <c r="E44" s="5"/>
+      <c r="E44" s="11">
+        <v>183.9</v>
+      </c>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A45" s="2">
@@ -1160,7 +1250,9 @@
       <c r="D45" s="3">
         <v>133</v>
       </c>
-      <c r="E45" s="3"/>
+      <c r="E45" s="10">
+        <v>188</v>
+      </c>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A46" s="4">
@@ -1175,7 +1267,9 @@
       <c r="D46" s="5">
         <v>20</v>
       </c>
-      <c r="E46" s="5"/>
+      <c r="E46" s="11">
+        <v>192.7</v>
+      </c>
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A47" s="2">
@@ -1190,7 +1284,9 @@
       <c r="D47" s="3">
         <v>163</v>
       </c>
-      <c r="E47" s="3"/>
+      <c r="E47" s="10">
+        <v>196.1</v>
+      </c>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A48" s="4">
@@ -1205,7 +1301,9 @@
       <c r="D48" s="5">
         <v>51</v>
       </c>
-      <c r="E48" s="5"/>
+      <c r="E48" s="11">
+        <v>200</v>
+      </c>
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A49" s="2">
@@ -1220,7 +1318,9 @@
       <c r="D49" s="3">
         <v>194</v>
       </c>
-      <c r="E49" s="3"/>
+      <c r="E49" s="10">
+        <v>203</v>
+      </c>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A50" s="4">
@@ -1235,7 +1335,9 @@
       <c r="D50" s="5">
         <v>81</v>
       </c>
-      <c r="E50" s="5"/>
+      <c r="E50" s="11">
+        <v>208</v>
+      </c>
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A51" s="2">
@@ -1250,7 +1352,9 @@
       <c r="D51" s="3">
         <v>225</v>
       </c>
-      <c r="E51" s="3"/>
+      <c r="E51" s="10">
+        <v>211</v>
+      </c>
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A52" s="4">
@@ -1265,7 +1369,9 @@
       <c r="D52" s="5">
         <v>112</v>
       </c>
-      <c r="E52" s="5"/>
+      <c r="E52" s="11">
+        <v>215</v>
+      </c>
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A53" s="2">
@@ -1280,7 +1386,9 @@
       <c r="D53" s="3">
         <v>0</v>
       </c>
-      <c r="E53" s="3"/>
+      <c r="E53" s="10">
+        <v>219</v>
+      </c>
     </row>
     <row r="54" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A54" s="4">
@@ -1295,7 +1403,9 @@
       <c r="D54" s="5">
         <v>143</v>
       </c>
-      <c r="E54" s="5"/>
+      <c r="E54" s="11">
+        <v>223</v>
+      </c>
     </row>
     <row r="55" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A55" s="2">
@@ -1310,7 +1420,9 @@
       <c r="D55" s="3">
         <v>30</v>
       </c>
-      <c r="E55" s="3"/>
+      <c r="E55" s="10">
+        <v>228</v>
+      </c>
     </row>
     <row r="56" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A56" s="4">
@@ -1325,7 +1437,9 @@
       <c r="D56" s="5">
         <v>174</v>
       </c>
-      <c r="E56" s="5"/>
+      <c r="E56" s="11">
+        <v>231</v>
+      </c>
     </row>
     <row r="57" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A57" s="2">
@@ -1340,7 +1454,9 @@
       <c r="D57" s="3">
         <v>61</v>
       </c>
-      <c r="E57" s="3"/>
+      <c r="E57" s="10">
+        <v>235</v>
+      </c>
     </row>
     <row r="58" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A58" s="4">
@@ -1355,7 +1471,9 @@
       <c r="D58" s="5">
         <v>204</v>
       </c>
-      <c r="E58" s="5"/>
+      <c r="E58" s="11">
+        <v>239</v>
+      </c>
     </row>
     <row r="59" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A59" s="2">
@@ -1370,7 +1488,9 @@
       <c r="D59" s="3">
         <v>92</v>
       </c>
-      <c r="E59" s="3"/>
+      <c r="E59" s="10">
+        <v>242</v>
+      </c>
     </row>
     <row r="60" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A60" s="4">
@@ -1385,7 +1505,9 @@
       <c r="D60" s="5">
         <v>235</v>
       </c>
-      <c r="E60" s="5"/>
+      <c r="E60" s="11">
+        <v>246</v>
+      </c>
     </row>
     <row r="61" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A61" s="2">
@@ -1400,7 +1522,9 @@
       <c r="D61" s="3">
         <v>122</v>
       </c>
-      <c r="E61" s="3"/>
+      <c r="E61" s="10">
+        <v>250</v>
+      </c>
     </row>
     <row r="62" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A62" s="4">
@@ -1415,7 +1539,9 @@
       <c r="D62" s="5">
         <v>10</v>
       </c>
-      <c r="E62" s="5"/>
+      <c r="E62" s="11">
+        <v>254</v>
+      </c>
     </row>
     <row r="63" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A63" s="2">
@@ -1430,7 +1556,9 @@
       <c r="D63" s="3">
         <v>153</v>
       </c>
-      <c r="E63" s="3"/>
+      <c r="E63" s="10">
+        <v>258</v>
+      </c>
     </row>
     <row r="64" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A64" s="4">
@@ -1445,7 +1573,9 @@
       <c r="D64" s="5">
         <v>40</v>
       </c>
-      <c r="E64" s="5"/>
+      <c r="E64" s="11">
+        <v>262</v>
+      </c>
     </row>
     <row r="65" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A65" s="2">
@@ -1460,7 +1590,9 @@
       <c r="D65" s="3">
         <v>184</v>
       </c>
-      <c r="E65" s="3"/>
+      <c r="E65" s="10">
+        <v>265</v>
+      </c>
     </row>
     <row r="66" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A66" s="4">
@@ -1475,7 +1607,9 @@
       <c r="D66" s="5">
         <v>71</v>
       </c>
-      <c r="E66" s="5"/>
+      <c r="E66" s="11">
+        <v>270</v>
+      </c>
     </row>
     <row r="67" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A67" s="2">
@@ -1490,7 +1624,9 @@
       <c r="D67" s="3">
         <v>214</v>
       </c>
-      <c r="E67" s="3"/>
+      <c r="E67" s="10">
+        <v>273</v>
+      </c>
     </row>
     <row r="68" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A68" s="4">
@@ -1505,7 +1641,9 @@
       <c r="D68" s="5">
         <v>102</v>
       </c>
-      <c r="E68" s="5"/>
+      <c r="E68" s="11">
+        <v>276</v>
+      </c>
     </row>
     <row r="69" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A69" s="2">
@@ -1520,7 +1658,9 @@
       <c r="D69" s="3">
         <v>245</v>
       </c>
-      <c r="E69" s="3"/>
+      <c r="E69" s="10">
+        <v>280</v>
+      </c>
     </row>
     <row r="70" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A70" s="4">
@@ -1535,7 +1675,9 @@
       <c r="D70" s="5">
         <v>132</v>
       </c>
-      <c r="E70" s="5"/>
+      <c r="E70" s="11">
+        <v>284</v>
+      </c>
     </row>
     <row r="71" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A71" s="2">
@@ -1550,7 +1692,9 @@
       <c r="D71" s="3">
         <v>20</v>
       </c>
-      <c r="E71" s="3"/>
+      <c r="E71" s="10">
+        <v>288</v>
+      </c>
     </row>
     <row r="72" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A72" s="4">
@@ -1565,7 +1709,9 @@
       <c r="D72" s="5">
         <v>163</v>
       </c>
-      <c r="E72" s="5"/>
+      <c r="E72" s="11">
+        <v>291</v>
+      </c>
     </row>
     <row r="73" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A73" s="2">
@@ -1580,7 +1726,9 @@
       <c r="D73" s="3">
         <v>50</v>
       </c>
-      <c r="E73" s="3"/>
+      <c r="E73" s="10">
+        <v>295</v>
+      </c>
     </row>
     <row r="74" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A74" s="4">
@@ -1595,7 +1743,9 @@
       <c r="D74" s="5">
         <v>194</v>
       </c>
-      <c r="E74" s="5"/>
+      <c r="E74" s="11">
+        <v>299</v>
+      </c>
     </row>
     <row r="75" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A75" s="2">
@@ -1610,7 +1760,9 @@
       <c r="D75" s="3">
         <v>81</v>
       </c>
-      <c r="E75" s="3"/>
+      <c r="E75" s="10">
+        <v>304</v>
+      </c>
     </row>
     <row r="76" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A76" s="4">
@@ -1625,7 +1777,9 @@
       <c r="D76" s="5">
         <v>225</v>
       </c>
-      <c r="E76" s="5"/>
+      <c r="E76" s="11">
+        <v>306</v>
+      </c>
     </row>
     <row r="77" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A77" s="2">
@@ -1640,7 +1794,9 @@
       <c r="D77" s="3">
         <v>112</v>
       </c>
-      <c r="E77" s="3"/>
+      <c r="E77" s="10">
+        <v>309</v>
+      </c>
     </row>
     <row r="78" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A78" s="4">
@@ -1655,7 +1811,9 @@
       <c r="D78" s="5">
         <v>255</v>
       </c>
-      <c r="E78" s="5"/>
+      <c r="E78" s="11">
+        <v>313</v>
+      </c>
     </row>
     <row r="79" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A79" s="2">
@@ -1670,7 +1828,9 @@
       <c r="D79" s="3">
         <v>143</v>
       </c>
-      <c r="E79" s="3"/>
+      <c r="E79" s="10">
+        <v>316</v>
+      </c>
     </row>
     <row r="80" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A80" s="4">
@@ -1685,7 +1845,9 @@
       <c r="D80" s="5">
         <v>30</v>
       </c>
-      <c r="E80" s="5"/>
+      <c r="E80" s="11">
+        <v>320</v>
+      </c>
     </row>
     <row r="81" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A81" s="2">
@@ -1700,7 +1862,9 @@
       <c r="D81" s="3">
         <v>173</v>
       </c>
-      <c r="E81" s="3"/>
+      <c r="E81" s="10">
+        <v>324</v>
+      </c>
     </row>
     <row r="82" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A82" s="4">
@@ -1715,7 +1879,9 @@
       <c r="D82" s="5">
         <v>61</v>
       </c>
-      <c r="E82" s="5"/>
+      <c r="E82" s="11">
+        <v>327</v>
+      </c>
     </row>
     <row r="83" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A83" s="2">
@@ -1730,7 +1896,9 @@
       <c r="D83" s="3">
         <v>204</v>
       </c>
-      <c r="E83" s="3"/>
+      <c r="E83" s="10">
+        <v>330</v>
+      </c>
     </row>
     <row r="84" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A84" s="4">
@@ -1745,7 +1913,9 @@
       <c r="D84" s="5">
         <v>91</v>
       </c>
-      <c r="E84" s="5"/>
+      <c r="E84" s="11">
+        <v>334</v>
+      </c>
     </row>
     <row r="85" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A85" s="2">
@@ -1760,7 +1930,9 @@
       <c r="D85" s="3">
         <v>235</v>
       </c>
-      <c r="E85" s="3"/>
+      <c r="E85" s="10">
+        <v>338</v>
+      </c>
     </row>
     <row r="86" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A86" s="4">
@@ -1775,7 +1947,9 @@
       <c r="D86" s="5">
         <v>122</v>
       </c>
-      <c r="E86" s="5"/>
+      <c r="E86" s="11">
+        <v>341</v>
+      </c>
     </row>
     <row r="87" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A87" s="2">
@@ -1790,7 +1964,9 @@
       <c r="D87" s="3">
         <v>9</v>
       </c>
-      <c r="E87" s="3"/>
+      <c r="E87" s="10">
+        <v>344</v>
+      </c>
     </row>
     <row r="88" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A88" s="4">
@@ -1805,7 +1981,9 @@
       <c r="D88" s="5">
         <v>153</v>
       </c>
-      <c r="E88" s="5"/>
+      <c r="E88" s="11">
+        <v>348</v>
+      </c>
     </row>
     <row r="89" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A89" s="2">
@@ -1820,7 +1998,9 @@
       <c r="D89" s="3">
         <v>40</v>
       </c>
-      <c r="E89" s="3"/>
+      <c r="E89" s="10">
+        <v>351</v>
+      </c>
     </row>
     <row r="90" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A90" s="4">
@@ -1835,7 +2015,9 @@
       <c r="D90" s="5">
         <v>183</v>
       </c>
-      <c r="E90" s="5"/>
+      <c r="E90" s="11">
+        <v>355</v>
+      </c>
     </row>
     <row r="91" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A91" s="2">
@@ -1850,7 +2032,9 @@
       <c r="D91" s="3">
         <v>71</v>
       </c>
-      <c r="E91" s="3"/>
+      <c r="E91" s="10">
+        <v>358</v>
+      </c>
     </row>
     <row r="92" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A92" s="4">
@@ -1865,7 +2049,9 @@
       <c r="D92" s="5">
         <v>214</v>
       </c>
-      <c r="E92" s="5"/>
+      <c r="E92" s="11">
+        <v>362</v>
+      </c>
     </row>
     <row r="93" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A93" s="2">
@@ -1880,7 +2066,9 @@
       <c r="D93" s="3">
         <v>102</v>
       </c>
-      <c r="E93" s="3"/>
+      <c r="E93" s="10">
+        <v>366</v>
+      </c>
     </row>
     <row r="94" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A94" s="4">
@@ -1895,7 +2083,9 @@
       <c r="D94" s="5">
         <v>245</v>
       </c>
-      <c r="E94" s="5"/>
+      <c r="E94" s="11">
+        <v>369</v>
+      </c>
     </row>
     <row r="95" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A95" s="2">
@@ -1910,7 +2100,9 @@
       <c r="D95" s="3">
         <v>132</v>
       </c>
-      <c r="E95" s="3"/>
+      <c r="E95" s="10">
+        <v>373</v>
+      </c>
     </row>
     <row r="96" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A96" s="4">
@@ -1925,7 +2117,9 @@
       <c r="D96" s="5">
         <v>20</v>
       </c>
-      <c r="E96" s="5"/>
+      <c r="E96" s="11">
+        <v>376</v>
+      </c>
     </row>
     <row r="97" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A97" s="2">
@@ -1940,7 +2134,9 @@
       <c r="D97" s="3">
         <v>163</v>
       </c>
-      <c r="E97" s="3"/>
+      <c r="E97" s="10">
+        <v>380</v>
+      </c>
     </row>
     <row r="98" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A98" s="4">
@@ -1955,7 +2151,9 @@
       <c r="D98" s="5">
         <v>50</v>
       </c>
-      <c r="E98" s="5"/>
+      <c r="E98" s="11">
+        <v>384</v>
+      </c>
     </row>
     <row r="99" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A99" s="2">
@@ -1970,7 +2168,9 @@
       <c r="D99" s="3">
         <v>194</v>
       </c>
-      <c r="E99" s="3"/>
+      <c r="E99" s="10">
+        <v>388</v>
+      </c>
     </row>
     <row r="100" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A100" s="4">
@@ -1985,7 +2185,9 @@
       <c r="D100" s="5">
         <v>81</v>
       </c>
-      <c r="E100" s="5"/>
+      <c r="E100" s="11">
+        <v>391</v>
+      </c>
     </row>
     <row r="101" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A101" s="2">
@@ -2000,7 +2202,9 @@
       <c r="D101" s="3">
         <v>224</v>
       </c>
-      <c r="E101" s="3"/>
+      <c r="E101" s="10">
+        <v>395</v>
+      </c>
     </row>
     <row r="102" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A102" s="4">
@@ -2015,7 +2219,9 @@
       <c r="D102" s="5">
         <v>112</v>
       </c>
-      <c r="E102" s="5"/>
+      <c r="E102" s="11">
+        <v>399</v>
+      </c>
     </row>
     <row r="103" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A103" s="2">
@@ -2030,13 +2236,16 @@
       <c r="D103" s="3">
         <v>255</v>
       </c>
-      <c r="E103" s="3"/>
+      <c r="E103" s="10">
+        <v>404</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:E1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>